<commit_message>
Fix Ktalé/Jezzine mohafaza typo: Mount Lebanon -> South (and DistrictTranslation Jezzine row)
</commit_message>
<xml_diff>
--- a/FuzzyMatch/Grok 4.6/Lebanese_Villages_Improved_Matching_v5.xlsx
+++ b/FuzzyMatch/Grok 4.6/Lebanese_Villages_Improved_Matching_v5.xlsx
@@ -22671,7 +22671,7 @@
       </c>
       <c r="D827" s="6" t="inlineStr">
         <is>
-          <t>Mount Lebanon</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E827" s="6" t="inlineStr">
@@ -85747,7 +85747,7 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Mount Lebanon</t>
+          <t>South</t>
         </is>
       </c>
     </row>

</xml_diff>